<commit_message>
Investor: founder salary £4k/month in model and deck; slide 15 seed-round wording matches model
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01D3BUwhgUWaWyPGkQWqj7G2
</commit_message>
<xml_diff>
--- a/jobstracker/investor/JobsTracker_Financial_Model_2026-10-18.xlsx
+++ b/jobstracker/investor/JobsTracker_Financial_Model_2026-10-18.xlsx
@@ -280,19 +280,19 @@
     <t xml:space="preserve">Legal, finance, contingency, £ per month — Option A</t>
   </si>
   <si>
-    <t xml:space="preserve">£120k over 15 months less hosting (modelled separately)</t>
+    <t xml:space="preserve">£60k over 15 months less hosting (modelled separately)</t>
   </si>
   <si>
     <t xml:space="preserve">Legal, finance, contingency, £ per month — Option B</t>
   </si>
   <si>
-    <t xml:space="preserve">£170k over 15 months less hosting</t>
+    <t xml:space="preserve">£110k over 15 months less hosting</t>
   </si>
   <si>
     <t xml:space="preserve">Founder salary, £ per year</t>
   </si>
   <si>
-    <t xml:space="preserve">Not in the use of funds on the deck; set a figure if the round will pay one</t>
+    <t xml:space="preserve">Franck: £4,000 a month from close; £60k over the 15-month budget on deck slide 16</t>
   </si>
   <si>
     <t xml:space="preserve">SCALING WITH VOLUME (drives years 2–3; the deck says a seed round in year 2 funds them)</t>
@@ -3538,7 +3538,7 @@
         <v>84</v>
       </c>
       <c r="B36" s="17" t="n">
-        <v>6500</v>
+        <v>2500</v>
       </c>
       <c r="C36" s="2"/>
       <c r="D36" s="13" t="s">
@@ -3585,7 +3585,7 @@
         <v>86</v>
       </c>
       <c r="B37" s="17" t="n">
-        <v>9500</v>
+        <v>5500</v>
       </c>
       <c r="C37" s="2"/>
       <c r="D37" s="13" t="s">
@@ -3631,8 +3631,8 @@
       <c r="A38" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="B38" s="19" t="n">
-        <v>0</v>
+      <c r="B38" s="17" t="n">
+        <v>48000</v>
       </c>
       <c r="C38" s="2"/>
       <c r="D38" s="13" t="s">
@@ -7677,147 +7677,147 @@
       </c>
       <c r="B26" s="11" t="n">
         <f aca="false">Assumptions!$B$36</f>
-        <v>6500</v>
+        <v>2500</v>
       </c>
       <c r="C26" s="11" t="n">
         <f aca="false">Assumptions!$B$36</f>
-        <v>6500</v>
+        <v>2500</v>
       </c>
       <c r="D26" s="11" t="n">
         <f aca="false">Assumptions!$B$36</f>
-        <v>6500</v>
+        <v>2500</v>
       </c>
       <c r="E26" s="11" t="n">
         <f aca="false">Assumptions!$B$36</f>
-        <v>6500</v>
+        <v>2500</v>
       </c>
       <c r="F26" s="11" t="n">
         <f aca="false">Assumptions!$B$36</f>
-        <v>6500</v>
+        <v>2500</v>
       </c>
       <c r="G26" s="11" t="n">
         <f aca="false">Assumptions!$B$36</f>
-        <v>6500</v>
+        <v>2500</v>
       </c>
       <c r="H26" s="11" t="n">
         <f aca="false">Assumptions!$B$36</f>
-        <v>6500</v>
+        <v>2500</v>
       </c>
       <c r="I26" s="11" t="n">
         <f aca="false">Assumptions!$B$36</f>
-        <v>6500</v>
+        <v>2500</v>
       </c>
       <c r="J26" s="11" t="n">
         <f aca="false">Assumptions!$B$36</f>
-        <v>6500</v>
+        <v>2500</v>
       </c>
       <c r="K26" s="11" t="n">
         <f aca="false">Assumptions!$B$36</f>
-        <v>6500</v>
+        <v>2500</v>
       </c>
       <c r="L26" s="11" t="n">
         <f aca="false">Assumptions!$B$36</f>
-        <v>6500</v>
+        <v>2500</v>
       </c>
       <c r="M26" s="11" t="n">
         <f aca="false">Assumptions!$B$36</f>
-        <v>6500</v>
+        <v>2500</v>
       </c>
       <c r="N26" s="11" t="n">
         <f aca="false">Assumptions!$B$36</f>
-        <v>6500</v>
+        <v>2500</v>
       </c>
       <c r="O26" s="11" t="n">
         <f aca="false">Assumptions!$B$36</f>
-        <v>6500</v>
+        <v>2500</v>
       </c>
       <c r="P26" s="11" t="n">
         <f aca="false">Assumptions!$B$36</f>
-        <v>6500</v>
+        <v>2500</v>
       </c>
       <c r="Q26" s="11" t="n">
         <f aca="false">Assumptions!$B$36</f>
-        <v>6500</v>
+        <v>2500</v>
       </c>
       <c r="R26" s="11" t="n">
         <f aca="false">Assumptions!$B$36</f>
-        <v>6500</v>
+        <v>2500</v>
       </c>
       <c r="S26" s="11" t="n">
         <f aca="false">Assumptions!$B$36</f>
-        <v>6500</v>
+        <v>2500</v>
       </c>
       <c r="T26" s="11" t="n">
         <f aca="false">Assumptions!$B$36</f>
-        <v>6500</v>
+        <v>2500</v>
       </c>
       <c r="U26" s="11" t="n">
         <f aca="false">Assumptions!$B$36</f>
-        <v>6500</v>
+        <v>2500</v>
       </c>
       <c r="V26" s="11" t="n">
         <f aca="false">Assumptions!$B$36</f>
-        <v>6500</v>
+        <v>2500</v>
       </c>
       <c r="W26" s="11" t="n">
         <f aca="false">Assumptions!$B$36</f>
-        <v>6500</v>
+        <v>2500</v>
       </c>
       <c r="X26" s="11" t="n">
         <f aca="false">Assumptions!$B$36</f>
-        <v>6500</v>
+        <v>2500</v>
       </c>
       <c r="Y26" s="11" t="n">
         <f aca="false">Assumptions!$B$36</f>
-        <v>6500</v>
+        <v>2500</v>
       </c>
       <c r="Z26" s="11" t="n">
         <f aca="false">Assumptions!$B$36</f>
-        <v>6500</v>
+        <v>2500</v>
       </c>
       <c r="AA26" s="11" t="n">
         <f aca="false">Assumptions!$B$36</f>
-        <v>6500</v>
+        <v>2500</v>
       </c>
       <c r="AB26" s="11" t="n">
         <f aca="false">Assumptions!$B$36</f>
-        <v>6500</v>
+        <v>2500</v>
       </c>
       <c r="AC26" s="11" t="n">
         <f aca="false">Assumptions!$B$36</f>
-        <v>6500</v>
+        <v>2500</v>
       </c>
       <c r="AD26" s="11" t="n">
         <f aca="false">Assumptions!$B$36</f>
-        <v>6500</v>
+        <v>2500</v>
       </c>
       <c r="AE26" s="11" t="n">
         <f aca="false">Assumptions!$B$36</f>
-        <v>6500</v>
+        <v>2500</v>
       </c>
       <c r="AF26" s="11" t="n">
         <f aca="false">Assumptions!$B$36</f>
-        <v>6500</v>
+        <v>2500</v>
       </c>
       <c r="AG26" s="11" t="n">
         <f aca="false">Assumptions!$B$36</f>
-        <v>6500</v>
+        <v>2500</v>
       </c>
       <c r="AH26" s="11" t="n">
         <f aca="false">Assumptions!$B$36</f>
-        <v>6500</v>
+        <v>2500</v>
       </c>
       <c r="AI26" s="11" t="n">
         <f aca="false">Assumptions!$B$36</f>
-        <v>6500</v>
+        <v>2500</v>
       </c>
       <c r="AJ26" s="11" t="n">
         <f aca="false">Assumptions!$B$36</f>
-        <v>6500</v>
+        <v>2500</v>
       </c>
       <c r="AK26" s="11" t="n">
         <f aca="false">Assumptions!$B$36</f>
-        <v>6500</v>
+        <v>2500</v>
       </c>
       <c r="AL26" s="2"/>
     </row>
@@ -7827,147 +7827,147 @@
       </c>
       <c r="B27" s="11" t="n">
         <f aca="false">Assumptions!$B$38/12</f>
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="C27" s="11" t="n">
         <f aca="false">Assumptions!$B$38/12</f>
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="D27" s="11" t="n">
         <f aca="false">Assumptions!$B$38/12</f>
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="E27" s="11" t="n">
         <f aca="false">Assumptions!$B$38/12</f>
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="F27" s="11" t="n">
         <f aca="false">Assumptions!$B$38/12</f>
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="G27" s="11" t="n">
         <f aca="false">Assumptions!$B$38/12</f>
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="H27" s="11" t="n">
         <f aca="false">Assumptions!$B$38/12</f>
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="I27" s="11" t="n">
         <f aca="false">Assumptions!$B$38/12</f>
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="J27" s="11" t="n">
         <f aca="false">Assumptions!$B$38/12</f>
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="K27" s="11" t="n">
         <f aca="false">Assumptions!$B$38/12</f>
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="L27" s="11" t="n">
         <f aca="false">Assumptions!$B$38/12</f>
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="M27" s="11" t="n">
         <f aca="false">Assumptions!$B$38/12</f>
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="N27" s="11" t="n">
         <f aca="false">Assumptions!$B$38/12</f>
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="O27" s="11" t="n">
         <f aca="false">Assumptions!$B$38/12</f>
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="P27" s="11" t="n">
         <f aca="false">Assumptions!$B$38/12</f>
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="Q27" s="11" t="n">
         <f aca="false">Assumptions!$B$38/12</f>
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="R27" s="11" t="n">
         <f aca="false">Assumptions!$B$38/12</f>
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="S27" s="11" t="n">
         <f aca="false">Assumptions!$B$38/12</f>
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="T27" s="11" t="n">
         <f aca="false">Assumptions!$B$38/12</f>
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="U27" s="11" t="n">
         <f aca="false">Assumptions!$B$38/12</f>
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="V27" s="11" t="n">
         <f aca="false">Assumptions!$B$38/12</f>
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="W27" s="11" t="n">
         <f aca="false">Assumptions!$B$38/12</f>
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="X27" s="11" t="n">
         <f aca="false">Assumptions!$B$38/12</f>
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="Y27" s="11" t="n">
         <f aca="false">Assumptions!$B$38/12</f>
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="Z27" s="11" t="n">
         <f aca="false">Assumptions!$B$38/12</f>
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="AA27" s="11" t="n">
         <f aca="false">Assumptions!$B$38/12</f>
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="AB27" s="11" t="n">
         <f aca="false">Assumptions!$B$38/12</f>
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="AC27" s="11" t="n">
         <f aca="false">Assumptions!$B$38/12</f>
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="AD27" s="11" t="n">
         <f aca="false">Assumptions!$B$38/12</f>
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="AE27" s="11" t="n">
         <f aca="false">Assumptions!$B$38/12</f>
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="AF27" s="11" t="n">
         <f aca="false">Assumptions!$B$38/12</f>
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="AG27" s="11" t="n">
         <f aca="false">Assumptions!$B$38/12</f>
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="AH27" s="11" t="n">
         <f aca="false">Assumptions!$B$38/12</f>
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="AI27" s="11" t="n">
         <f aca="false">Assumptions!$B$38/12</f>
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="AJ27" s="11" t="n">
         <f aca="false">Assumptions!$B$38/12</f>
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="AK27" s="11" t="n">
         <f aca="false">Assumptions!$B$38/12</f>
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="AL27" s="2"/>
     </row>
@@ -8197,11 +8197,11 @@
       </c>
       <c r="I30" s="11" t="n">
         <f aca="false">I18-I28</f>
-        <v>7387.14396169514</v>
+        <v>7387.14396169513</v>
       </c>
       <c r="J30" s="11" t="n">
         <f aca="false">J18-J28</f>
-        <v>18011.9391887448</v>
+        <v>18011.9391887449</v>
       </c>
       <c r="K30" s="11" t="n">
         <f aca="false">K18-K28</f>
@@ -11598,147 +11598,147 @@
       </c>
       <c r="B26" s="11" t="n">
         <f aca="false">Assumptions!$B$37</f>
-        <v>9500</v>
+        <v>5500</v>
       </c>
       <c r="C26" s="11" t="n">
         <f aca="false">Assumptions!$B$37</f>
-        <v>9500</v>
+        <v>5500</v>
       </c>
       <c r="D26" s="11" t="n">
         <f aca="false">Assumptions!$B$37</f>
-        <v>9500</v>
+        <v>5500</v>
       </c>
       <c r="E26" s="11" t="n">
         <f aca="false">Assumptions!$B$37</f>
-        <v>9500</v>
+        <v>5500</v>
       </c>
       <c r="F26" s="11" t="n">
         <f aca="false">Assumptions!$B$37</f>
-        <v>9500</v>
+        <v>5500</v>
       </c>
       <c r="G26" s="11" t="n">
         <f aca="false">Assumptions!$B$37</f>
-        <v>9500</v>
+        <v>5500</v>
       </c>
       <c r="H26" s="11" t="n">
         <f aca="false">Assumptions!$B$37</f>
-        <v>9500</v>
+        <v>5500</v>
       </c>
       <c r="I26" s="11" t="n">
         <f aca="false">Assumptions!$B$37</f>
-        <v>9500</v>
+        <v>5500</v>
       </c>
       <c r="J26" s="11" t="n">
         <f aca="false">Assumptions!$B$37</f>
-        <v>9500</v>
+        <v>5500</v>
       </c>
       <c r="K26" s="11" t="n">
         <f aca="false">Assumptions!$B$37</f>
-        <v>9500</v>
+        <v>5500</v>
       </c>
       <c r="L26" s="11" t="n">
         <f aca="false">Assumptions!$B$37</f>
-        <v>9500</v>
+        <v>5500</v>
       </c>
       <c r="M26" s="11" t="n">
         <f aca="false">Assumptions!$B$37</f>
-        <v>9500</v>
+        <v>5500</v>
       </c>
       <c r="N26" s="11" t="n">
         <f aca="false">Assumptions!$B$37</f>
-        <v>9500</v>
+        <v>5500</v>
       </c>
       <c r="O26" s="11" t="n">
         <f aca="false">Assumptions!$B$37</f>
-        <v>9500</v>
+        <v>5500</v>
       </c>
       <c r="P26" s="11" t="n">
         <f aca="false">Assumptions!$B$37</f>
-        <v>9500</v>
+        <v>5500</v>
       </c>
       <c r="Q26" s="11" t="n">
         <f aca="false">Assumptions!$B$37</f>
-        <v>9500</v>
+        <v>5500</v>
       </c>
       <c r="R26" s="11" t="n">
         <f aca="false">Assumptions!$B$37</f>
-        <v>9500</v>
+        <v>5500</v>
       </c>
       <c r="S26" s="11" t="n">
         <f aca="false">Assumptions!$B$37</f>
-        <v>9500</v>
+        <v>5500</v>
       </c>
       <c r="T26" s="11" t="n">
         <f aca="false">Assumptions!$B$37</f>
-        <v>9500</v>
+        <v>5500</v>
       </c>
       <c r="U26" s="11" t="n">
         <f aca="false">Assumptions!$B$37</f>
-        <v>9500</v>
+        <v>5500</v>
       </c>
       <c r="V26" s="11" t="n">
         <f aca="false">Assumptions!$B$37</f>
-        <v>9500</v>
+        <v>5500</v>
       </c>
       <c r="W26" s="11" t="n">
         <f aca="false">Assumptions!$B$37</f>
-        <v>9500</v>
+        <v>5500</v>
       </c>
       <c r="X26" s="11" t="n">
         <f aca="false">Assumptions!$B$37</f>
-        <v>9500</v>
+        <v>5500</v>
       </c>
       <c r="Y26" s="11" t="n">
         <f aca="false">Assumptions!$B$37</f>
-        <v>9500</v>
+        <v>5500</v>
       </c>
       <c r="Z26" s="11" t="n">
         <f aca="false">Assumptions!$B$37</f>
-        <v>9500</v>
+        <v>5500</v>
       </c>
       <c r="AA26" s="11" t="n">
         <f aca="false">Assumptions!$B$37</f>
-        <v>9500</v>
+        <v>5500</v>
       </c>
       <c r="AB26" s="11" t="n">
         <f aca="false">Assumptions!$B$37</f>
-        <v>9500</v>
+        <v>5500</v>
       </c>
       <c r="AC26" s="11" t="n">
         <f aca="false">Assumptions!$B$37</f>
-        <v>9500</v>
+        <v>5500</v>
       </c>
       <c r="AD26" s="11" t="n">
         <f aca="false">Assumptions!$B$37</f>
-        <v>9500</v>
+        <v>5500</v>
       </c>
       <c r="AE26" s="11" t="n">
         <f aca="false">Assumptions!$B$37</f>
-        <v>9500</v>
+        <v>5500</v>
       </c>
       <c r="AF26" s="11" t="n">
         <f aca="false">Assumptions!$B$37</f>
-        <v>9500</v>
+        <v>5500</v>
       </c>
       <c r="AG26" s="11" t="n">
         <f aca="false">Assumptions!$B$37</f>
-        <v>9500</v>
+        <v>5500</v>
       </c>
       <c r="AH26" s="11" t="n">
         <f aca="false">Assumptions!$B$37</f>
-        <v>9500</v>
+        <v>5500</v>
       </c>
       <c r="AI26" s="11" t="n">
         <f aca="false">Assumptions!$B$37</f>
-        <v>9500</v>
+        <v>5500</v>
       </c>
       <c r="AJ26" s="11" t="n">
         <f aca="false">Assumptions!$B$37</f>
-        <v>9500</v>
+        <v>5500</v>
       </c>
       <c r="AK26" s="11" t="n">
         <f aca="false">Assumptions!$B$37</f>
-        <v>9500</v>
+        <v>5500</v>
       </c>
       <c r="AL26" s="2"/>
     </row>
@@ -11748,147 +11748,147 @@
       </c>
       <c r="B27" s="11" t="n">
         <f aca="false">Assumptions!$B$38/12</f>
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="C27" s="11" t="n">
         <f aca="false">Assumptions!$B$38/12</f>
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="D27" s="11" t="n">
         <f aca="false">Assumptions!$B$38/12</f>
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="E27" s="11" t="n">
         <f aca="false">Assumptions!$B$38/12</f>
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="F27" s="11" t="n">
         <f aca="false">Assumptions!$B$38/12</f>
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="G27" s="11" t="n">
         <f aca="false">Assumptions!$B$38/12</f>
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="H27" s="11" t="n">
         <f aca="false">Assumptions!$B$38/12</f>
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="I27" s="11" t="n">
         <f aca="false">Assumptions!$B$38/12</f>
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="J27" s="11" t="n">
         <f aca="false">Assumptions!$B$38/12</f>
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="K27" s="11" t="n">
         <f aca="false">Assumptions!$B$38/12</f>
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="L27" s="11" t="n">
         <f aca="false">Assumptions!$B$38/12</f>
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="M27" s="11" t="n">
         <f aca="false">Assumptions!$B$38/12</f>
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="N27" s="11" t="n">
         <f aca="false">Assumptions!$B$38/12</f>
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="O27" s="11" t="n">
         <f aca="false">Assumptions!$B$38/12</f>
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="P27" s="11" t="n">
         <f aca="false">Assumptions!$B$38/12</f>
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="Q27" s="11" t="n">
         <f aca="false">Assumptions!$B$38/12</f>
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="R27" s="11" t="n">
         <f aca="false">Assumptions!$B$38/12</f>
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="S27" s="11" t="n">
         <f aca="false">Assumptions!$B$38/12</f>
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="T27" s="11" t="n">
         <f aca="false">Assumptions!$B$38/12</f>
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="U27" s="11" t="n">
         <f aca="false">Assumptions!$B$38/12</f>
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="V27" s="11" t="n">
         <f aca="false">Assumptions!$B$38/12</f>
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="W27" s="11" t="n">
         <f aca="false">Assumptions!$B$38/12</f>
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="X27" s="11" t="n">
         <f aca="false">Assumptions!$B$38/12</f>
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="Y27" s="11" t="n">
         <f aca="false">Assumptions!$B$38/12</f>
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="Z27" s="11" t="n">
         <f aca="false">Assumptions!$B$38/12</f>
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="AA27" s="11" t="n">
         <f aca="false">Assumptions!$B$38/12</f>
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="AB27" s="11" t="n">
         <f aca="false">Assumptions!$B$38/12</f>
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="AC27" s="11" t="n">
         <f aca="false">Assumptions!$B$38/12</f>
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="AD27" s="11" t="n">
         <f aca="false">Assumptions!$B$38/12</f>
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="AE27" s="11" t="n">
         <f aca="false">Assumptions!$B$38/12</f>
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="AF27" s="11" t="n">
         <f aca="false">Assumptions!$B$38/12</f>
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="AG27" s="11" t="n">
         <f aca="false">Assumptions!$B$38/12</f>
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="AH27" s="11" t="n">
         <f aca="false">Assumptions!$B$38/12</f>
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="AI27" s="11" t="n">
         <f aca="false">Assumptions!$B$38/12</f>
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="AJ27" s="11" t="n">
         <f aca="false">Assumptions!$B$38/12</f>
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="AK27" s="11" t="n">
         <f aca="false">Assumptions!$B$38/12</f>
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="AL27" s="2"/>
     </row>

</xml_diff>